<commit_message>
AI RMF question banks: full run (Sonnet generator, Opus evaluator)
Foundation 31 subcategories (84 questions; 2 need human review: GOVERN 4.2, 5.1).
Areas 41 subcategories (202 questions; 6 need human review: MAP 3.5, MAP 4.1,
MEASURE 2.4, MEASURE 2.10, MANAGE 4.1, MANAGE 4.3). Both banks current.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ai/authoring/questions_foundation.xlsx
+++ b/data/ai/authoring/questions_foundation.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Read me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Foundation questions'!$A$1:$K$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Foundation questions'!$A$1:$K$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -508,12 +508,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 1.2</t>
+          <t>GOVERN 1.1</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>The characteristics of trustworthy AI are integrated into organizational policies, processes, and procedures.</t>
+          <t>Legal and regulatory requirements involving AI are understood, managed, and documented.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -523,18 +523,18 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>none, consumer, producer</t>
+          <t>consumer, producer</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Where is your AI risk management policy kept, and how do the people it applies to (staff, developers, vendors' account owners) come to know it and any changes to it, for example through onboarding, training, acknowledgement or announcements?</t>
+          <t>Where are the legal and regulatory requirements that apply to your use or building of AI kept, and how do the people they apply to learn of them and of changes (for example onboarding, training, announcements)?</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 1.2 — suggested action 2, GOVERN 1.2 — suggested action 14</t>
+          <t>GOVERN 1.1 — suggested action 1, GOVERN 1.1 — suggested action 3</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -546,19 +546,19 @@
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>agent</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 1.2</t>
+          <t>GOVERN 1.1</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>The characteristics of trustworthy AI are integrated into organizational policies, processes, and procedures.</t>
+          <t>Legal and regulatory requirements involving AI are understood, managed, and documented.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -574,12 +574,12 @@
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>How do your AI rules apply to AI that others built or sold to you, as well as AI you run yourself, so that it meets your existing legal obligations and risk controls? Who checks this?</t>
+          <t>How does your organisation keep track of new or changing laws and regulations that affect its AI? Who decides what must change in how AI is used or built?</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 1.2 — suggested action 13, GOVERN 1.2 — suggested action 15</t>
+          <t>GOVERN 1.1 — suggested action 1, GOVERN 1.1 — suggested action 2</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -591,7 +591,7 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>agent</t>
         </is>
       </c>
     </row>
@@ -608,23 +608,23 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>consumer, producer</t>
+          <t>none, consumer, producer</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>What do your procedures require to happen before an AI system goes live and while it is in use (testing and validation, legal and risk review, ongoing monitoring), and what record shows these steps were followed for a recent AI system?</t>
+          <t>Where is your AI risk management policy kept, and how do the people it applies to (staff, developers, vendors' account owners) come to know it and any changes to it, for example through onboarding, training, acknowledgement or announcements?</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 1.2 — suggested action 6, GOVERN 1.2 — suggested action 7, GOVERN 1.2 — suggested action 8</t>
+          <t>GOVERN 1.2 — suggested action 2, GOVERN 1.2 — suggested action 14</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -653,7 +653,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -664,12 +664,12 @@
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>How do your AI policies and procedures address qualities such as safety, security, fairness, explainability and privacy for your AI systems, and where can we see this applied to a recent AI system?</t>
+          <t>How do your AI rules apply to AI that others built or sold to you, as well as AI you run yourself, so that it meets your existing legal obligations and risk controls? Who checks this?</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 1.2 — suggested action 14</t>
+          <t>GOVERN 1.2 — suggested action 13, GOVERN 1.2 — suggested action 15</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -698,23 +698,23 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>producer</t>
+          <t>consumer, producer</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>How do your rules for building and training your own models set standards for data quality and model training? Where can we see them applied to your latest model?</t>
+          <t>What do your procedures require to happen before an AI system goes live and while it is in use (testing and validation, legal and risk review, ongoing monitoring), and what record shows these steps were followed for a recent AI system?</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 1.2 — suggested action 4</t>
+          <t>GOVERN 1.2 — suggested action 6, GOVERN 1.2 — suggested action 7, GOVERN 1.2 — suggested action 8</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -733,17 +733,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 1.6</t>
+          <t>GOVERN 1.2</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Mechanisms are in place to inventory AI systems and are resourced according to organizational risk priorities.</t>
+          <t>The characteristics of trustworthy AI are integrated into organizational policies, processes, and procedures.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -754,12 +754,12 @@
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>In the 'AI systems' sheet, list each AI system your organisation uses or builds, with what it involves and the worst realistic outcome if it gets things wrong.</t>
+          <t>How do your AI policies and procedures address qualities such as safety, security, fairness, explainability and privacy for your AI systems, and where can we see this applied to a recent AI system?</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 1.6 — suggested action 3, GOVERN 1.6 — suggested action 4</t>
+          <t>GOVERN 1.2 — suggested action 14</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -778,33 +778,33 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 1.6</t>
+          <t>GOVERN 1.2</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Mechanisms are in place to inventory AI systems and are resourced according to organizational risk priorities.</t>
+          <t>The characteristics of trustworthy AI are integrated into organizational policies, processes, and procedures.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>consumer, producer</t>
+          <t>producer</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>How does a new or changed AI system get added to your AI system inventory, and who is responsible for that?</t>
+          <t>How do your rules for building and training your own models set standards for data quality and model training? Where can we see them applied to your latest model?</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 1.6 — suggested action 1, GOVERN 1.6 — suggested action 2</t>
+          <t>GOVERN 1.2 — suggested action 4</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -823,17 +823,17 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 1.6</t>
+          <t>GOVERN 1.3</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Mechanisms are in place to inventory AI systems and are resourced according to organizational risk priorities.</t>
+          <t>Processes and procedures are in place to determine the needed level of risk management activities based on the organization's risk tolerance.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -844,12 +844,12 @@
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>How does an AI system's criticality decide how much goes into its inventory entry — which details are recorded and how often it is reviewed — and where is that shown?</t>
+          <t>How do you decide how much risk assessment and oversight an AI system needs before it is used, for example using a risk rating of its possible impact and likelihood? Who makes that decision?</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 1.6 — suggested action 3, GOVERN 1.6 — suggested action 4</t>
+          <t>GOVERN 1.3 — suggested action 1, GOVERN 1.3 — suggested action 4</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -861,24 +861,24 @@
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>agent</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 6.1</t>
+          <t>GOVERN 1.3</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Policies and procedures are in place that address AI risks associated with third-party entities, including risks of infringement of a third party’s intellectual property or other rights.</t>
+          <t>Processes and procedures are in place to determine the needed level of risk management activities based on the organization's risk tolerance.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -889,12 +889,12 @@
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Where are your rules for using third-party AI (models, AI services and the data they rely on) kept, and how do the people they apply to come to know them and any changes, for example through onboarding, training or announcements?</t>
+          <t>How are your AI systems placed on one common risk scale? How often is that rating revisited as the system or its use changes?</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 6.1 — suggested action 1, GOVERN 6.1 — suggested action 7</t>
+          <t>GOVERN 1.3 — suggested action 3, GOVERN 1.3 — suggested action 5</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -913,17 +913,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 6.1</t>
+          <t>GOVERN 1.4</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Policies and procedures are in place that address AI risks associated with third-party entities, including risks of infringement of a third party’s intellectual property or other rights.</t>
+          <t>The risk management process and its outcomes are established through transparent policies, procedures, and other controls based on organizational risk priorities.</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -934,12 +934,12 @@
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Before your organisation starts using a third-party AI system or data source, how is it checked for what it does, what it was trained on and its known limits, for example through vendor documentation and your own testing? Who signs off?</t>
+          <t>What information do you record about each AI system, for example its purpose, limits, known risks and test results? Where are these records kept?</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 6.1 — suggested action 3, GOVERN 6.1 — suggested action 4, GOVERN 6.1 — suggested action 5</t>
+          <t>GOVERN 1.4 — suggested action 1, GOVERN 1.4 — suggested action 16</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -958,17 +958,17 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 6.1</t>
+          <t>GOVERN 1.4</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Policies and procedures are in place that address AI risks associated with third-party entities, including risks of infringement of a third party’s intellectual property or other rights.</t>
+          <t>The risk management process and its outcomes are established through transparent policies, procedures, and other controls based on organizational risk priorities.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -979,12 +979,12 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>How do you check that third-party AI and the data it was built on do not infringe someone else's intellectual property or other rights, for example through contract terms or licence reviews? Where is the outcome recorded?</t>
+          <t>How often do you check whether your AI risk management process is working? Who is responsible for acting on what the check finds?</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 6.1 — suggested action 2, GOVERN 6.1 — suggested action 7</t>
+          <t>GOVERN 1.4 — suggested action 17, GOVERN 1.4 — suggested action 18</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -1003,17 +1003,17 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 6.1</t>
+          <t>GOVERN 1.4</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Policies and procedures are in place that address AI risks associated with third-party entities, including risks of infringement of a third party’s intellectual property or other rights.</t>
+          <t>The risk management process and its outcomes are established through transparent policies, procedures, and other controls based on organizational risk priorities.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1024,12 +1024,12 @@
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>How are your rules for third-party AI reviewed and updated, for example after a vendor change, an incident or a new law? Who owns that review?</t>
+          <t>How do you decide what to tell customers, regulators or the public about your use of AI and its risks, and who approves what is shared?</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 6.1 — suggested action 6</t>
+          <t>GOVERN 1.4 — suggested action 19</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -1048,37 +1048,33 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 6.1</t>
+          <t>GOVERN 1.4</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Policies and procedures are in place that address AI risks associated with third-party entities, including risks of infringement of a third party’s intellectual property or other rights.</t>
+          <t>The risk management process and its outcomes are established through transparent policies, procedures, and other controls based on organizational risk priorities.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>producer</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>built_on_existing_model</t>
-        </is>
-      </c>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>How do you choose, check and keep watching the existing model your own model is built on, for example its source, licence and known weaknesses? Who owns this?</t>
+          <t>Where are your AI risk management policies and procedures kept, and how do the people they apply to come to know them and their changes (for example onboarding, training, announcements)?</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>GOVERN 6.1 — suggested action 3, GOVERN 6.1 — suggested action 4</t>
+          <t>GOVERN 1.4 — suggested action 1, GOVERN 1.4 — suggested action 15</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -1094,10 +1090,3221 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.5</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Ongoing monitoring and periodic review of the risk management process and its outcomes are planned, organizational roles and responsibilities are clearly defined, including determining the frequency of periodic review.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>How are your AI systems monitored after they go live for performance, bias and security problems? What record shows the latest results?</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.5 — suggested action 2</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.5</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Ongoing monitoring and periodic review of the risk management process and its outcomes are planned, organizational roles and responsibilities are clearly defined, including determining the frequency of periodic review.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Where is your procedure for handling AI incidents kept, and how do the people involved come to know it and its changes (for example training, drills, announcements)?</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.5 — suggested action 3</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.5</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Ongoing monitoring and periodic review of the risk management process and its outcomes are planned, organizational roles and responsibilities are clearly defined, including determining the frequency of periodic review.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Which roles or teams are responsible for monitoring your AI and responding to AI incidents, and where is that assignment written down?</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.5 — suggested action 4</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.5</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Ongoing monitoring and periodic review of the risk management process and its outcomes are planned, organizational roles and responsibilities are clearly defined, including determining the frequency of periodic review.</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>How often do you review the results of your AI monitoring and incidents to decide whether your AI risk management needs to change? Who carries out the review?</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.5 — suggested action 2, GOVERN 1.5 — suggested action 4</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.6</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Mechanisms are in place to inventory AI systems and are resourced according to organizational risk priorities.</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>In the 'AI systems' sheet, list each AI system your organisation uses or builds, with what it involves and the worst realistic outcome if it gets things wrong.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.6 — suggested action 3, GOVERN 1.6 — suggested action 4</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.6</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Mechanisms are in place to inventory AI systems and are resourced according to organizational risk priorities.</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>How does a new or changed AI system get added to your AI system inventory, and who is responsible for that?</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.6 — suggested action 1, GOVERN 1.6 — suggested action 2</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.6</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Mechanisms are in place to inventory AI systems and are resourced according to organizational risk priorities.</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>How does an AI system's criticality decide how much goes into its inventory entry — which details are recorded and how often it is reviewed — and where is that shown?</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.6 — suggested action 3, GOVERN 1.6 — suggested action 4</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.7</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Processes and procedures are in place for decommissioning and phasing out of AI systems safely and in a manner that does not increase risks or decrease the organization’s trustworthiness.</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>When an AI system is retired or replaced, how do you carry it out safely, for example moving to the replacement and checking what depends on it? Who signs it off?</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.7 — suggested action 1, GOVERN 1.7 — suggested action 7, GOVERN 1.7 — suggested action 4</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.7</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Processes and procedures are in place for decommissioning and phasing out of AI systems safely and in a manner that does not increase risks or decrease the organization’s trustworthiness.</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>What happens to the models, data and records of a retired AI system, and for how long are they kept?</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.7 — suggested action 8, GOVERN 1.7 — suggested action 10</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.7</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Processes and procedures are in place for decommissioning and phasing out of AI systems safely and in a manner that does not increase risks or decrease the organization’s trustworthiness.</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Where is your procedure for retiring AI systems kept, and how do the people it applies to come to know it and its changes (for example onboarding, training, announcements)?</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 1.7 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 2.1</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Roles and responsibilities and lines of communication related to mapping, measuring, and managing AI risks are documented and are clear to individuals and teams throughout the organization.</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Who is responsible for AI risk in your organisation, from senior management to the teams that buy, build, test and run AI, and where are these responsibilities written down? How do people learn who to go to?</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 2.1 — suggested action 1, GOVERN 2.1 — suggested action 3</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 2.1</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Roles and responsibilities and lines of communication related to mapping, measuring, and managing AI risks are documented and are clear to individuals and teams throughout the organization.</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>How do the people involved in AI risk talk to each other and raise concerns, for example regular meetings or an escalation route? What record shows it happening?</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 2.1 — suggested action 14</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 2.1</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Roles and responsibilities and lines of communication related to mapping, measuring, and managing AI risks are documented and are clear to individuals and teams throughout the organization.</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>How do you keep the people who check or approve an AI system independent of the people who built or bought it? Where are conflicts of interest declared or recorded?</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 2.1 — suggested action 15, GOVERN 2.1 — suggested action 16</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 2.2</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>The organization’s personnel and partners receive AI risk management training to enable them to perform their duties and responsibilities consistent with related policies, procedures, and agreements.</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>What AI risk training do your staff and partners get, for example on laws, AI policies and possible harms? How does it differ for technical and oversight roles?</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 2.2 — suggested action 1, GOVERN 2.2 — suggested action 6</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 2.2</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>The organization’s personnel and partners receive AI risk management training to enable them to perform their duties and responsibilities consistent with related policies, procedures, and agreements.</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>How do staff acknowledge their AI responsibilities and learn of significant changes to AI systems or policies?</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 2.2 — suggested action 8, GOVERN 2.2 — suggested action 9</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 2.2</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>The organization’s personnel and partners receive AI risk management training to enable them to perform their duties and responsibilities consistent with related policies, procedures, and agreements.</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Who do staff and partners escalate AI risk concerns to, and how do they know that route?</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 2.2 — suggested action 10</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 2.3</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Executive leadership of the organization takes responsibility for decisions about risks associated with AI system development and deployment.</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>How does executive leadership decide how much AI risk the organisation will accept? Where is that decision recorded?</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 2.3 — suggested action 2, GOVERN 2.3 — suggested action 5</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 2.3</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Executive leadership of the organization takes responsibility for decisions about risks associated with AI system development and deployment.</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>How often does leadership or a board committee review AI risks and approve decisions on high-risk AI use? What record, such as minutes or a report, shows this?</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 2.3 — suggested action 3, GOVERN 2.3 — suggested action 7</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 3.1</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Decision-makings related to mapping, measuring, and managing AI risks throughout the lifecycle is informed by a diverse team (e.g., diversity of demographics, disciplines, experience, expertise, and backgrounds).</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>How do you make sure the people who decide on AI risks bring different disciplines and backgrounds, for example legal, security, business and technical staff? Where is who took part recorded?</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 3.1 — suggested action 1, GOVERN 3.1 — suggested action 2</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 3.1</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Decision-makings related to mapping, measuring, and managing AI risks throughout the lifecycle is informed by a diverse team (e.g., diversity of demographics, disciplines, experience, expertise, and backgrounds).</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>When your organisation lacks expertise on AI risk, how do you bring in outside help? Who decides when it is needed?</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 3.1 — suggested action 4</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 3.2</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Policies and procedures are in place to define and differentiate roles and responsibilities for human-AI configurations and oversight of AI systems.</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Where are the roles and responsibilities of the people who use, oversee or monitor your AI systems written down, and how do those people come to know them and any changes?</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 3.2 — suggested action 1, GOVERN 3.2 — suggested action 5</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 3.2</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Policies and procedures are in place to define and differentiate roles and responsibilities for human-AI configurations and oversight of AI systems.</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>How do you train and check the skills of the people who operate or oversee your AI systems? Who owns this?</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 3.2 — suggested action 3, GOVERN 3.2 — suggested action 4</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 3.2</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Policies and procedures are in place to define and differentiate roles and responsibilities for human-AI configurations and oversight of AI systems.</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>How are problems in the way people work with AI, such as over-reliance on its answers or confusing screens, captured and tracked? Where are they recorded?</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 3.2 — suggested action 2, GOVERN 3.2 — suggested action 8</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 4.1</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Organizational policies, and practices are in place to foster a critical thinking and safety-first mindset in the design, development, deployment, and uses of AI systems to minimize negative impacts.</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>At what point in an AI project do legal, compliance and risk staff get involved, and what shows they were (for example a sign-off or review record)?</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 4.1 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 4.1</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Organizational policies, and practices are in place to foster a critical thinking and safety-first mindset in the design, development, deployment, and uses of AI systems to minimize negative impacts.</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>How are decisions to build or deploy AI challenged before they go ahead, for example by an independent review, audit or red-teaming? Who carries out the challenge?</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 4.1 — suggested action 2, GOVERN 4.1 — suggested action 3</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 4.1</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Organizational policies, and practices are in place to foster a critical thinking and safety-first mindset in the design, development, deployment, and uses of AI systems to minimize negative impacts.</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>How can staff raise a concern about an AI system without fear of reprisal? Where are concerns recorded?</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 4.1 — suggested action 4</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 4.2</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Organizational teams document the risks and potential impacts of the AI technology they design, develop, deploy, evaluate and use, and communicate about the impacts more broadly.</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr"/>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>How do you assess the potential harm of an AI system before it is used and again when it changes? Who carries out the assessment?</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 4.2 — suggested action 1, GOVERN 4.2 — suggested action 3</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Whole subcategory: The outcome's second half, communicating the impacts more broadly beyond the team, is no longer asked by any question (question 2 now only asks internal use).</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 4.2</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Organizational teams document the risks and potential impacts of the AI technology they design, develop, deploy, evaluate and use, and communicate about the impacts more broadly.</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Where are the results of these assessments recorded, and how are they used in your wider view of AI risk?</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 4.2 — suggested action 2, GOVERN 4.2 — suggested action 4</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Whole subcategory: The outcome's second half, communicating the impacts more broadly beyond the team, is no longer asked by any question (question 2 now only asks internal use).</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 4.3</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Organizational practices are in place to enable AI testing, identification of incidents, and information sharing.</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>How are your AI systems tested before and during use? Where are the results kept?</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 4.3 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 4.3</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Organizational practices are in place to enable AI testing, identification of incidents, and information sharing.</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Where are the steps for reporting and handling an AI incident kept, and how do staff come to know them and any changes?</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 4.3 — suggested action 3, GOVERN 4.3 — suggested action 5</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 4.3</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Organizational practices are in place to enable AI testing, identification of incidents, and information sharing.</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr"/>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>How do you share what you learn about the limits of your AI systems and about incidents, inside the organisation and with outside parties where needed? Who decides what is shared?</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 4.3 — suggested action 2, GOVERN 4.3 — suggested action 4</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 5.1</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Organizational policies and practices are in place to collect, consider, prioritize, and integrate feedback from those external to the team that developed or deployed the AI system regarding the potential individual and societal impacts related to AI risks.</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>How do you collect feedback about your AI from people outside the team that runs it, such as users, customers or people affected by it? Where is it recorded?</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 5.1 — suggested action 1, GOVERN 5.1 — suggested action 6</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 5.1</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Organizational policies and practices are in place to collect, consider, prioritize, and integrate feedback from those external to the team that developed or deployed the AI system regarding the potential individual and societal impacts related to AI risks.</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>How is that outside feedback reviewed and prioritised, and who decides what is changed as a result?</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 5.1 — suggested action 7</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr"/>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 5.1</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Organizational policies and practices are in place to collect, consider, prioritize, and integrate feedback from those external to the team that developed or deployed the AI system regarding the potential individual and societal impacts related to AI risks.</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>How do you tell customers, partners and the public the principles that guide your use of AI? Where are they published?</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 5.1 — suggested action 8</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>check 4: Publishing AI principles informs outsiders of the org's values; it does not test collecting, considering, prioritising or integrating external feedback, which is this outcome.</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 5.2</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Mechanisms are established to enable AI actors to regularly incorporate adjudicated feedback from relevant AI actors into system design and implementation.</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr"/>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Who is given the chance to give feedback on how an AI system is designed or set up (for example the people who build, run, use or oversee it), and how is that feedback gathered?</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 5.2 — suggested action 3</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 5.2</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Mechanisms are established to enable AI actors to regularly incorporate adjudicated feedback from relevant AI actors into system design and implementation.</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>When feedback on an AI system is received, how is it weighed and accepted or rejected before anything changes? Who decides?</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 5.2 — suggested action 3</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 5.2</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Mechanisms are established to enable AI actors to regularly incorporate adjudicated feedback from relevant AI actors into system design and implementation.</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>How does feedback from the people who use or are affected by an AI system lead to changes in how it is designed or run? Can you give a recent example?</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 5.2 — suggested action 3</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr"/>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 6.1</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Policies and procedures are in place that address AI risks associated with third-party entities, including risks of infringement of a third party’s intellectual property or other rights.</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Where are your rules for using third-party AI (models, AI services and the data they rely on) kept, and how do the people they apply to come to know them and any changes, for example through onboarding, training or announcements?</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 6.1 — suggested action 1, GOVERN 6.1 — suggested action 7</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 6.1</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Policies and procedures are in place that address AI risks associated with third-party entities, including risks of infringement of a third party’s intellectual property or other rights.</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr"/>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Before your organisation starts using a third-party AI system or data source, how is it checked for what it does, what it was trained on and its known limits, for example through vendor documentation and your own testing? Who signs off?</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 6.1 — suggested action 3, GOVERN 6.1 — suggested action 4, GOVERN 6.1 — suggested action 5</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr"/>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr"/>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 6.1</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Policies and procedures are in place that address AI risks associated with third-party entities, including risks of infringement of a third party’s intellectual property or other rights.</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>How do you check that third-party AI and the data it was built on do not infringe someone else's intellectual property or other rights, for example through contract terms or licence reviews? Where is the outcome recorded?</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 6.1 — suggested action 2, GOVERN 6.1 — suggested action 7</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 6.1</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Policies and procedures are in place that address AI risks associated with third-party entities, including risks of infringement of a third party’s intellectual property or other rights.</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr"/>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>How are your rules for third-party AI reviewed and updated, for example after a vendor change, an incident or a new law? Who owns that review?</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 6.1 — suggested action 6</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr"/>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 6.1</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Policies and procedures are in place that address AI risks associated with third-party entities, including risks of infringement of a third party’s intellectual property or other rights.</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>producer</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>built_on_existing_model</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>How do you choose, check and keep watching the existing model your own model is built on, for example its source, licence and known weaknesses? Who owns this?</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 6.1 — suggested action 3, GOVERN 6.1 — suggested action 4</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr"/>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 6.2</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Contingency processes are in place to handle failures or incidents in third-party data or AI systems deemed to be high-risk.</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>How does your incident response plan cover a failure or incident in a third-party AI service or data source you rely on? Who owns that part of the plan?</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 6.2 — suggested action 2</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr"/>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 6.2</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Contingency processes are in place to handle failures or incidents in third-party data or AI systems deemed to be high-risk.</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>For the third-party AI services you cannot do without, what backup exists (for example another provider or a manual process)? Who decided it was enough?</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>GOVERN 6.2 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>MAP 1.3</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>The organization’s mission and relevant goals for the AI technology are understood and documented.</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>How does your organisation record what each AI system it uses or builds is for, in light of its mission and goals? Who owns that record?</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>MAP 1.3 — suggested action 5</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr"/>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>MAP 1.3</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>The organization’s mission and relevant goals for the AI technology are understood and documented.</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>When the purpose of an AI system is reviewed, how are the organisation's stated principles and the values of the people affected taken into account, and where is the outcome recorded?</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>MAP 1.3 — suggested action 2, MAP 1.3 — suggested action 3</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>MAP 1.5</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Organizational risk tolerances are determined and documented.</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr"/>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>How does your organisation decide how much risk it will accept from AI, for example by type of harm and by level of impact? Where are these limits recorded?</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>MAP 1.5 — suggested action 2, MAP 1.5 — suggested action 3</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>MAP 1.5</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Organizational risk tolerances are determined and documented.</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>What happens when an AI system goes beyond the risk your organisation is willing to accept, or is used for a purpose it was not approved for? Can you give a recent example and the record of the decision?</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>MAP 1.5 — suggested action 4, MAP 1.5 — suggested action 6</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>MAP 3.4</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Processes for operator and practitioner proficiency with AI system performance and trustworthiness – and relevant technical standards and certifications – are defined, assessed and documented.</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr"/>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>How does your organisation decide what skills and training people need before they operate AI systems? Where are the training records kept?</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>MAP 3.4 — suggested action 2, MAP 3.4 — suggested action 3, MAP 3.4 — suggested action 4</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr"/>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>MAP 3.4</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Processes for operator and practitioner proficiency with AI system performance and trustworthiness – and relevant technical standards and certifications – are defined, assessed and documented.</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>How do you tell the people who use your AI systems what the systems can and cannot do, and what is out of bounds? Where do they find this information?</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>MAP 3.4 — suggested action 1, MAP 3.4 — suggested action 3, MAP 3.4 — suggested action 4</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 1.1</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Approaches and metrics for measurement of AI risks enumerated during the Map function are selected for implementation starting with the most significant AI risks. The risks or trustworthiness characteristics that will not – or cannot – be measured are properly documented.</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr"/>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>How does your organisation choose which AI risks to measure first? Where are the chosen measures recorded?</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 1.1 — suggested action 1, MEASURE 1.1 — suggested action 2, MEASURE 1.1 — suggested action 8</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr"/>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 1.1</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Approaches and metrics for measurement of AI risks enumerated during the Map function are selected for implementation starting with the most significant AI risks. The risks or trustworthiness characteristics that will not – or cannot – be measured are properly documented.</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>How are AI risks you decided not to measure, or cannot yet measure, recorded, and who accepted that decision?</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 1.1 — suggested action 12</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr"/>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 1.1</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Approaches and metrics for measurement of AI risks enumerated during the Map function are selected for implementation starting with the most significant AI risks. The risks or trustworthiness characteristics that will not – or cannot – be measured are properly documented.</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr"/>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>What happens when an AI system performs beyond the acceptable limits you have set for it, for example on error rates? Where is the decision recorded?</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 1.1 — suggested action 4</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr"/>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr"/>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 1.2</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Appropriateness of AI metrics and effectiveness of existing controls is regularly assessed and updated including reports of errors and impacts on affected communities.</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr"/>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>How often does your organisation check whether its AI measures and controls still work? Who does it?</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 1.2 — suggested action 2, MEASURE 1.2 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr"/>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 1.2</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Appropriateness of AI metrics and effectiveness of existing controls is regularly assessed and updated including reports of errors and impacts on affected communities.</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr"/>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>When errors, incidents or harm from AI are reported, how are they recorded and used to change the measures or controls? Can you show a recent example?</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 1.2 — suggested action 3, MEASURE 1.2 — suggested action 4, MEASURE 1.2 — suggested action 7</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr"/>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 3.1</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Approaches, personnel, and documentation are in place to regularly identify and track existing, unanticipated, and emergent AI risks based on factors such as intended and actual performance in deployed contexts.</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>How does your organisation track AI risks that appear after an AI system is in use, including ones nobody expected? Where is this recorded?</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 3.1 — suggested action 6</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 3.1</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Approaches, personnel, and documentation are in place to regularly identify and track existing, unanticipated, and emergent AI risks based on factors such as intended and actual performance in deployed contexts.</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr"/>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>How is feedback from users and affected people about AI compared with your own measures of how the AI performs? Where is the comparison recorded?</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 3.1 — suggested action 5</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr"/>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr"/>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 3.2</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Risk tracking approaches are considered for settings where AI risks are difficult to assess using currently available measurement techniques or where metrics are not yet available.</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>For AI risks that are hard to measure, how does your organisation keep track of them anyway, for example through user feedback, a way to challenge AI outputs, or testing by outsiders? Who is responsible?</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 3.2 — suggested action 1, MEASURE 3.2 — suggested action 2</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr"/>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr"/>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 3.2</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Risk tracking approaches are considered for settings where AI risks are difficult to assess using currently available measurement techniques or where metrics are not yet available.</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr"/>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>How does the organisation weigh AI risks that cannot be measured when deciding to approve, change or stop an AI system? Where is that decision recorded?</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 3.2 — suggested action 8, MEASURE 3.2 — suggested action 12</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr"/>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr"/>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 4.1</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Measurement approaches for identifying AI risks are connected to deployment context(s) and informed through consultation with domain experts and other end users. Approaches are documented.</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>How does your organisation collect feedback from the people who use AI systems about how well the AI works in their daily tasks? Where is it recorded?</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 4.1 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr"/>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 4.1</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Measurement approaches for identifying AI risks are connected to deployment context(s) and informed through consultation with domain experts and other end users. Approaches are documented.</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr"/>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>How does feedback from the people who use your AI systems lead to changes in how you measure AI risk? Can you show a recent change that came from it?</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>MEASURE 4.1 — suggested action 10, MEASURE 4.1 — suggested action 11</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr"/>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr"/>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 1.2</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Treatment of documented AI risks is prioritized based on impact, likelihood, or available resources or methods.</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>How does your organisation decide which AI risks get treated first and with the most oversight? Who makes these decisions?</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 1.2 — suggested action 1, MANAGE 1.2 — suggested action 2</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr"/>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 1.2</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Treatment of documented AI risks is prioritized based on impact, likelihood, or available resources or methods.</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr"/>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>How often are priorities and risk limits for AI reviewed, and what triggers an earlier review? Can you show the last one?</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 1.2 — suggested action 3</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr"/>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 1.3</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Responses to the AI risks deemed high priority as identified by the Map function, are developed, planned, and documented. Risk response options can include mitigating, transferring, avoiding, or accepting.</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>For the AI risks you rate as high priority, how does your organisation decide the response (reduce, transfer, avoid or accept)? Who owns each plan?</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 1.3 — suggested action 2, MANAGE 1.3 — suggested action 4</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr"/>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 1.3</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Responses to the AI risks deemed high priority as identified by the Map function, are developed, planned, and documented. Risk response options can include mitigating, transferring, avoiding, or accepting.</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr"/>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Where are AI risk responses and system documentation kept, and who can access them?</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 1.3 — suggested action 5</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr"/>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr"/>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 1.4</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Negative residual risks (defined as the sum of all unmitigated risks) to both downstream acquirers of AI systems and end users are documented.</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr"/>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>How does your organisation document the risks that remain after its AI risk controls are in place? Who accepts them?</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 1.4 — suggested action 1</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr"/>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr"/>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 1.4</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Negative residual risks (defined as the sum of all unmitigated risks) to both downstream acquirers of AI systems and end users are documented.</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr"/>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>How do you tell the people who rely on your AI systems (customers, staff, or those who receive them from you) about remaining risks, known limits and safe-use requirements? Where is this communicated?</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 1.4 — suggested action 2, MANAGE 1.4 — suggested action 3</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr"/>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr"/>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 2.1</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Resources required to manage AI risks are taken into account, along with viable non-AI alternative systems, approaches, or methods – to reduce the magnitude or likelihood of potential impacts.</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>When your organisation plans to use AI, how does it check that it has the staff, skills and budget to manage the risks? Who decides?</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 2.1 — suggested action 1, MANAGE 2.1 — suggested action 2</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr"/>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr"/>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 2.1</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Resources required to manage AI risks are taken into account, along with viable non-AI alternative systems, approaches, or methods – to reduce the magnitude or likelihood of potential impacts.</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr"/>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>Before choosing an AI system, how do you consider a non-AI or manual alternative, and where is that decision recorded?</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 2.1 — suggested action 3</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr"/>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr"/>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 2.1</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Resources required to manage AI risks are taken into account, along with viable non-AI alternative systems, approaches, or methods – to reduce the magnitude or likelihood of potential impacts.</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>How do you use past AI failures and negative impacts to avoid repeating them? Can you show a recent example?</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 2.1 — suggested action 6</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr"/>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr"/>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 2.1</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Resources required to manage AI risks are taken into account, along with viable non-AI alternative systems, approaches, or methods – to reduce the magnitude or likelihood of potential impacts.</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>consumer, producer</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr"/>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>Where your own team lacks the expertise to manage AI risks, how do you bring in outside expertise? Can you show a recent example?</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>MANAGE 2.1 — suggested action 12</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr"/>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr"/>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K14"/>
+  <autoFilter ref="A1:K85"/>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I214" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="I2:I285" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"pass,needs_human_review"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>